<commit_message>
docs(tracker): add Bug Log sheet to the Testing epic
Consolidates every defect the testing effort has surfaced into one trackable
place (previously only in commit messages + individual backlog-row notes).

Bug Log sheet: 10 findings -> 3 Fixed (operating-score crash, dedup float
tolerance, payment double-allocation), 6 Flagged as founder product decisions
(negative amounts, negative remaining, unassigned-task double-count, operations
default perms, None<->70 discontinuity, unparseable-date dup), 1 Disproven
(the blank-due_date "inconsistency" -- both modules actually guard it). Plus 4
test-infra/wiring items (3 fixed stale/lost-file issues + 1 open pre-existing
stale grep-test). Each row carries severity, status, fix commit, the pinning
test, and the scenario id.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,8 +72,28 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F2937"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00374151"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -104,6 +125,11 @@
         <fgColor rgb="00F3F4F6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -131,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -164,6 +190,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -10260,4 +10293,755 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Epic 10 -- Bug Log</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Defects surfaced by the testing effort (Sprint 1 unit + Sprint 8/10/11 DB tests). Every bug is pinned by a passing test; 'Fixed' rows link the fix commit, 'Flagged' rows are product decisions left to the founder, 'Disproven' rows were checked and are not bugs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>Tally: 10 findings -&gt; 3 Fixed, 6 Flagged (product decisions), 1 Disproven. Plus 4 test-infra/wiring items.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>Found</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F4" s="20" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Fix commit</t>
+        </is>
+      </c>
+      <c r="H4" s="20" t="inlineStr">
+        <is>
+          <t>Pinned by (test)</t>
+        </is>
+      </c>
+      <c r="I4" s="20" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>BUG-01</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Operating score</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Company-view did float(invoice.amount) with NO guard -&gt; a non-numeric OR OCR-formatted amount ('N/A', 'Rs 5,000') raised ValueError and crashed the ENTIRE operating score for the tenant.</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>e8d9b3c</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>test_s1_operating_score_view_unit.py</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>T10-07.14</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>BUG-02</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Finance / dedup</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Duplicate detection compared amounts with exact float == , so float-rounding (0.1+0.2 vs 0.3) escaped the amount-window rule.</t>
+        </is>
+      </c>
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>e8d9b3c</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>test_s1_finance_math_unit.py</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>T10-07.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>BUG-03</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Finance / payments</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>_apply_payment_to_invoice was read-modify-write with NO CAS: two payments reconciling one invoice from a stale snapshot both allocated the full balance (double-allocation / lost update).</t>
+        </is>
+      </c>
+      <c r="F7" s="21" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>ed49c23</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>test_s10_payment_concurrency.py</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>T10-10.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>BUG-04</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Finance / parse</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>parse_amount accepts negative money ('-500' -&gt; -500.0), which flows unclamped into outstanding / net_profit.</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>Flagged (product decision: credit notes / adjustments may be legitimate)</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>test_s1_finance_math_unit.py</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>T10-07.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>BUG-05</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Finance / ledger</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>_remaining goes negative on overpayment (no floor); negative remaining feeds contact/revenue outstanding sums.</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>Flagged (product decision: negative = real overpayment credit; flooring would hide it)</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>test_s1_finance_math_unit.py</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>T10-07.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>BUG-06</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Operating score</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>An unassigned role-only task is credited to EVERY member of that role in _score_employees -&gt; N-way double-count of 'done'.</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Flagged (product decision: is a shared role task everyone's or no one's?)</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>test_s1_operating_score_unit.py</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>T10-07.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>BUG-07</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>RBAC / permissions</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>The 'operations' role is canonical + in DEFAULT_ROLES but has NO ROLE_DEFAULT_PERMS entry -&gt; silently falls back to base perms (no people/finance/ledger).</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Flagged (product decision: what should ops see by default?)</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>test_s1_permissions_matrix_unit.py</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>T10-03.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>BUG-08</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Operating score</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>Company overall flips None&lt;-&gt;a number at exactly actionable 2-&gt;3 / inv_count 0-&gt;1 (new-tenant discontinuity); employee default 0 vs company 0.7 asymmetry.</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Flagged (product decision: unscored vs 70% for a data-thin tenant)</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>test_s1_operating_score_view_unit.py</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>T10-07.1 / T10-07.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>BUG-09</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Finance / dedup</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>_dup_reason: an unparseable date makes a same-amount same-vendor bill a duplicate regardless of how far apart.</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Flagged (defensible: conservative flagging routes to human review)</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>test_s1_finance_math_unit.py</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>T10-07.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>BUG-10</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Operating score vs finance_signals</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>Initial code-map flagged a blank-due_date 'overdue' inconsistency between operating_score and finance_signals.</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>Disproven by test: finance_signals._overdue_receivables ALSO guards blank dates (`if due and ...`) -&gt; both agree, no bug.</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>test_s1_operating_score_unit.py</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>T10-07.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>INF-01</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Test infra</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>test_tenant_deletion</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>KNOWN_TENANT_SCOPED_COLLECTIONS never picked up the brain_contexts-&gt;brain_query_cache rename -&gt; drift test red against the authoritative delete list.</t>
+        </is>
+      </c>
+      <c r="F15" s="21" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>89dd758</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>test_tenant_deletion.py</t>
+        </is>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>INF-02</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Test infra</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>test_operating_score_role_split</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>Stale source-grep test read server.py for functions the Epic 8 refactor moved to routers/services operating_score.py.</t>
+        </is>
+      </c>
+      <c r="F16" s="21" t="inlineStr">
+        <is>
+          <t>Fixed (repointed)</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>e8d9b3c</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>test_operating_score_role_split.py</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>INF-03</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Wiring</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>S9 compliance</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>The S9 commit captured stale copies of 4 modified files (routing/schedulers/AdminPortal/baseline) -- compliance router was unregistered on HEAD.</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr">
+        <is>
+          <t>Fixed (recovered)</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>2929b47</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>test_api_parity.py</t>
+        </is>
+      </c>
+      <c r="I17" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>INF-04</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Test infra</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>test_brain_write_coverage</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>TestNewWriteSites greps server.py for the workflow-advance brain_context write (moved by the refactor) -&gt; 2 stale failures.</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>Open (pre-existing, unrelated to fixes above)</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>test_brain_write_coverage.py</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(tracker): log stale-test cleanup results + categorized remaining tail
Bug Log: INF-04 fixed; +INF-05 (39 stale failures -> green across 9 source-grep
suites), INF-06 (test_workflows_dynamic = event-loop harness bug, open),
INF-07 (tenancy/phone tail = mixed shim + possibly-real behavioural fake-DB
failures, flagged for investigation not blind-shimmed).

Backlog: T10-11.2 (fix pre-existing failures) + T10-11.8 (flaky triage) ->
In progress with the results.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -157,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -198,6 +198,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1110,6 +1111,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -8595,13 +8597,13 @@
       </c>
       <c r="I125" s="11" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="J125" s="11" t="n"/>
       <c r="K125" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>In progress: stale-test cleanup fixed 39 pre-existing failures across 9 source-grep suites (repointed to Epic-8 homes). Remaining: the iteration_* live suite (needs the isolated-DB backend) + test_workflows_dynamic event-loop harness (INF-06).</t>
         </is>
       </c>
       <c r="L125" s="11" t="inlineStr">
@@ -8931,13 +8933,13 @@
       </c>
       <c r="I131" s="11" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="J131" s="11" t="n"/>
       <c r="K131" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>In progress: triaged the 27 source-grep suites -&gt; 9 fixed. Remaining tail categorized in Bug Log INF-06 (event-loop harness) + INF-07 (mixed shim + possibly-real behavioural fake-DB failures).</t>
         </is>
       </c>
       <c r="L131" s="11" t="inlineStr">
@@ -10301,7 +10303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11020,24 +11022,165 @@
           <t>TestNewWriteSites greps server.py for the workflow-advance brain_context write (moved by the refactor) -&gt; 2 stale failures.</t>
         </is>
       </c>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>Open (pre-existing, unrelated to fixes above)</t>
+      <c r="F18" s="21" t="inlineStr">
+        <is>
+          <t>Fixed (repointed to services.workflow_engine.advance)</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
+          <t>5ef38b4</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>test_brain_write_coverage.py</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H18" s="12" t="inlineStr">
-        <is>
-          <t>test_brain_write_coverage.py</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr">
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>INF-05</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Test infra</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>stale-test cleanup (9 files)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Source-inspection tests grepped server.py for functions/routes/index code the Epic 8 refactor moved to routers/services/bootstrap. Repointed imports + getsource targets + a compat shim + the WE-07 writer allowlist.</t>
+        </is>
+      </c>
+      <c r="F19" s="22" t="inlineStr">
+        <is>
+          <t>Fixed (39 stale failures -&gt; green across 9 files)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>e518077/1d2d854/065732e/5ef38b4</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>test_audit_log, test_plans_and_ai_keys, test_rbac_wave3_role_model, test_session_revocation, test_we07, test_we_stage_version_init, test_brain_hygiene, test_brain_write_coverage, test_rbac_wave3_gates</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>T10-11.2 / T10-11.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>INF-06</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Test infra</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>test_workflows_dynamic</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>All 11 failures are 'Cannot use AsyncMongoClient in different event loop' -- the test reuses one async client across asyncio.run calls (Motor tolerated this; PyMongo AsyncMongoClient binds to one loop). A harness bug from the Motor-&gt;PyMongo-async migration, not stale-source and not a code bug.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Open -- needs async-harness rewrite (one-loop pattern, like conftest.with_test_db)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>test_workflows_dynamic.py</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>T10-11.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>INF-07</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Needs investigation</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>test_tenant_phone_routing + test_tenancy_hygiene_batch</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Remaining tail (8): a few more moved-fn shims/repoints (resolve_wa_tenant, whatsapp_logs, tenant_terminal_stages) PLUS behavioural fake-DB failures (resolve_wa_tenant returns a UUID not the expected tenant; tenant-scoped task lookup returns 0) that may be REAL regressions -- flagged for investigation, not blind-shimmed.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Open -- triage: separate the source-grep repoints from possibly-real behaviour</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>test_tenant_phone_routing.py, test_tenancy_hygiene_batch.py</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>T10-11.8</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(functional): Epic 10 Sprint 2 batch 1 -- operating-score views, inbox, contact cascade
db-tier functional flows (tests/test_s2_functional.py) driving the real handlers
against an isolated Mongo db:

  T10-02.14  operating-score viewer dispatch: owner->company(+my_snapshot),
             non-owner->self, owner ?user_id->target self-view+view_as, non-owner
             ?user_id->403, owner->ghost->404.
  T10-02.12  inbox list paginates but counts + open_total reflect the FULL open
             set; bad status->400, missing id->404.
  T10-02.4   contact rename cascades name into invoices/payments/workflows;
             outstanding splits purchase_bill->payables vs sales->receivables.

Full suite 1245 passed / 0 failed (+3). Sprint 2 now 3/14. No prod code changed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -2549,15 +2549,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I17" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I17" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J17" s="11" t="n"/>
       <c r="K17" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s2_functional.test_contact_rename_cascade_and_outstanding_split: rename cascades contact_name into invoices+payments and counterparty on workflows (by contact_id); outstanding_by_contact splits purchase_bill-&gt;payables (400) vs sales-&gt;receivables (1000).</t>
         </is>
       </c>
       <c r="L17" s="11" t="inlineStr">
@@ -2997,15 +2997,15 @@
           <t>S</t>
         </is>
       </c>
-      <c r="I25" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I25" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J25" s="11" t="n"/>
       <c r="K25" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s2_functional.test_inbox_counts_full_open_total_and_status_validation: list paginates (limit=2) but counts + open_total reflect the FULL open set (5, complaint=3/payment=2); bad status-&gt;400, missing id-&gt;404.</t>
         </is>
       </c>
       <c r="L25" s="11" t="inlineStr">
@@ -3109,15 +3109,15 @@
           <t>S</t>
         </is>
       </c>
-      <c r="I27" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I27" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J27" s="11" t="n"/>
       <c r="K27" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s2_functional.test_operating_score_viewer_dispatch_and_privacy: owner-&gt;company view(+my_snapshot), non-owner-&gt;self, owner ?user_id-&gt;target self-view+view_as, non-owner ?user_id-&gt;403 (privacy), owner-&gt;ghost-&gt;404.</t>
         </is>
       </c>
       <c r="L27" s="11" t="inlineStr">

</xml_diff>

<commit_message>
test(functional): Epic 10 Sprint 2 batch 2 -- complaint + workflow lifecycle
  T10-02.10  complaint log (open + auto-inbox) -> resolve (writes a resolution
             brain_context row) -> missing 404; memory write/read round-trip.
  T10-02.3   workflow create validates type (unknown->400, starts at stage[0]);
             advance with an open stage task->409; override without reason->400;
             audited override forces the transition.

Also hardened the db-tier helper: deep flows (workflow engine) touch several
modules' global db (core.deps.tenant_role_keys, brain_context, ...) -- each must
be pointed at the isolated db or it cross-loop-fails under the shared client /
hits founder-os-58. Enumerated them via the cross-loop traceback.

Full suite 1247 passed / 0 failed (+2). Sprint 2 now 5/14.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -2493,15 +2493,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I16" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I16" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J16" s="11" t="n"/>
       <c r="K16" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s2_functional.test_workflow_create_and_advance_gating: create validates type (unknown-&gt;400), starts at stage[0]; advance with an open stage task-&gt;409; override without reason-&gt;400; audited override (with reason) forces the transition.</t>
         </is>
       </c>
       <c r="L16" s="11" t="inlineStr">
@@ -2885,15 +2885,15 @@
           <t>S</t>
         </is>
       </c>
-      <c r="I23" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I23" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J23" s="11" t="n"/>
       <c r="K23" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s2_functional.test_complaint_log_resolve_and_memory: log (status open + auto-inbox), resolve writes a 'resolution' brain_context row, missing-&gt;404, memory write+read round-trips (write gated on brain).</t>
         </is>
       </c>
       <c r="L23" s="11" t="inlineStr">

</xml_diff>

<commit_message>
test(functional): Epic 10 Sprint 2 batch 3 -- decision approve/reject lifecycle
  T10-02.1  approve -> status approved, blocked tasks unblocked, procurement
            workflow auto-advances requested->approved, writes a decision
            brain_context row; reject -> status rejected, cascade-deletes
            tasks/workflows/calendar (NO orphans), dismisses inbox; missing->404.

db-tier helper now skips modules with no `db` global (services.workflows uses
call-time imports). Full suite 1248 passed / 0 failed (+1). Sprint 2 now 6/14.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -2381,15 +2381,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I14" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J14" s="11" t="n"/>
       <c r="K14" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s2_functional.test_decision_approve_and_reject_lifecycle: approve -&gt; status approved, blocked tasks unblocked (todo), procurement workflow auto-advances requested-&gt;approved, writes a 'decision' brain_context row; reject -&gt; status rejected, cascade-deletes tasks/workflows/calendar (NO orphans), dismisses the inbox item; missing decision -&gt; 404.</t>
         </is>
       </c>
       <c r="L14" s="11" t="inlineStr">

</xml_diff>

<commit_message>
test(functional): Epic 10 Sprint 2 batch 4 -- task lifecycle (T10-02.2)
Role task with no assignee auto-routes to the least-loaded member; evidence gate
blocks done without proof (400); unapproved task can't start (403); valid done ->
status done + progress 100; invalid status 400, missing 404; completing an
invoice-task auto-creates a draft invoice, idempotent by source_task_id.

Full suite 1249 passed / 0 failed (+2). Sprint 2 now 7/14.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -2437,15 +2437,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I15" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I15" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J15" s="11" t="n"/>
       <c r="K15" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s2_functional.test_task_gates_smart_route_and_auto_invoice: role task with no assignee auto-routes to the least-loaded member; evidence_required blocks done without proof (400); unapproved task can't start (403); valid done -&gt; status done + progress 100; invalid status 400, missing 404; completing an invoice-task auto-creates a draft invoice, idempotent by source_task_id.</t>
         </is>
       </c>
       <c r="L15" s="11" t="inlineStr">

</xml_diff>

<commit_message>
test(functional): Epic 10 Sprint 2 batch 5 -- leave request/approve + attendance (T10-02.11)
Unknown leave type->400, end-before-start->400, valid request->pending, approve
(leave_approve)->approved; attendance upserts one row per (user,date), latest
mark wins.

Full suite 1250 passed / 0 failed (+1). Sprint 2 now 8/14.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -2941,15 +2941,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I24" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I24" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J24" s="11" t="n"/>
       <c r="K24" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s2_functional.test_leave_request_validation_approve_and_attendance: unknown leave type-&gt;400, end-before-start-&gt;400, valid request-&gt;pending, approve (leave_approve)-&gt;approved; attendance upserts one row per (user,date) with latest-mark-wins.</t>
         </is>
       </c>
       <c r="L24" s="11" t="inlineStr">

</xml_diff>

<commit_message>
test(functional): Epic 10 Sprint 2 batch 6 -- WhatsApp webhook gates (T10-02.13)
Pure unit test: GET verify echoes the challenge only on mode+token match (else
403); POST with no WA_ACCESS_TOKEN is a JSON no-op; configured + signature
mismatch -> 403; prod without WA_APP_SECRET -> 503.

Full suite 1251 passed / 0 failed (+1). Sprint 2 now 9/14. Remaining 5 are the
AI/LLM-in-the-flow items (ingest, ledger-OCR, Ask, voice, meeting) needing the
provider mocked.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -3053,15 +3053,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I26" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I26" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J26" s="11" t="n"/>
       <c r="K26" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s2_functional.test_whatsapp_verify_and_webhook_gates: GET verify echoes challenge only on mode+token match (else 403); POST no WA_ACCESS_TOKEN-&gt;JSON no-op; configured+signature mismatch-&gt;403; prod without WA_APP_SECRET-&gt;503. (whatsapp_logs tenant-scoping pinned in test_tenant_phone_routing.)</t>
         </is>
       </c>
       <c r="L26" s="11" t="inlineStr">

</xml_diff>

<commit_message>
test(isolation): Epic 10 Sprint 8 batch 1 -- tenant deletion, WhatsApp logs, file serve
  T10-08.8  seed A+B in EVERY tenant-scoped collection, delete A -> 0 rows for A
            across all 30 collections + tenant doc gone, B fully intact; missing->404.
  T10-08.5  WhatsApp logs strictly tenant-scoped: owner of A sees only A's events,
            never tenant B's and never unrouted (tenant_id=None).
  T10-08.4  file serve-by-name: path traversal -> 404; a file owned by another
            tenant is not resolvable in the caller's scope -> 404.

Full suite 1260 passed / 0 failed (+3). Sprint 8 now 5/10.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -6917,15 +6917,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I95" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I95" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J95" s="11" t="n"/>
       <c r="K95" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s8_isolation_scenarios.test_file_serve_by_name_tenant_scope_and_traversal: path traversal (../, leading-dot, slash) -&gt; 404; a file owned by another tenant is not resolvable in the caller's scope -&gt; 404.</t>
         </is>
       </c>
       <c r="L95" s="11" t="inlineStr">
@@ -6973,15 +6973,15 @@
           <t>S</t>
         </is>
       </c>
-      <c r="I96" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I96" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J96" s="11" t="n"/>
       <c r="K96" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s8_isolation_scenarios.test_whatsapp_logs_hide_other_tenants_and_unrouted: owner of A sees ONLY A's wa_events -- never tenant B's, never unrouted (tenant_id=None) events.</t>
         </is>
       </c>
       <c r="L96" s="11" t="inlineStr">
@@ -7141,15 +7141,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I99" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I99" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J99" s="11" t="n"/>
       <c r="K99" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s8_isolation_scenarios.test_tenant_deletion_removes_A_and_keeps_B: seed A+B in EVERY TENANT_COLLECTIONS collection, delete A -&gt; 0 rows for A across all + tenant doc gone; B fully intact; missing tenant -&gt; 404.</t>
         </is>
       </c>
       <c r="L99" s="11" t="inlineStr">

</xml_diff>

<commit_message>
test(isolation): Epic 10 Sprint 8 batch 2 -- brain-doc visibility + uniqueness
  T10-08.6  _chunk_visible matrix: owner+team_manage & uploader see all;
            public->anyone; dept->matching dept or allow-listed role;
            private->allow-listed role only.
  T10-08.9  users.email globally unique (same email can't back a 2nd tenant's
            user); memberships (user_id,tenant_id) compound-unique, but a user
            CAN belong to two tenants.

Full suite 1262 passed / 0 failed (+2). Sprint 8 now 7/10.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -7029,15 +7029,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I97" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I97" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J97" s="11" t="n"/>
       <c r="K97" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s8_isolation_scenarios.test_brain_chunk_visibility_matrix: _chunk_visible matrix -- owner+team_manage &amp; uploader see all; public-&gt;anyone; dept-&gt;matching department or allow-listed role; private-&gt;allow-listed role only. A user can't see a doc they aren't cleared for.</t>
         </is>
       </c>
       <c r="L97" s="11" t="inlineStr">
@@ -7197,15 +7197,15 @@
           <t>S</t>
         </is>
       </c>
-      <c r="I100" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I100" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J100" s="11" t="n"/>
       <c r="K100" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s8_isolation_scenarios.test_email_global_unique_and_membership_compound_unique: users.email is globally unique (same email can't back a 2nd tenant's user); memberships are (user_id,tenant_id) compound-unique, but the same user CAN belong to two tenants.</t>
         </is>
       </c>
       <c r="L100" s="11" t="inlineStr">

</xml_diff>

<commit_message>
test(isolation): finish Epic 10 Sprint 8 -- auth guards + OTP tenant-keying (10/10)
  T10-08.3   legacy no-membership fallback is trusted only when the user's own
             tenant_id == the token's claimed tenant (no cross-tenant confusion).
  T10-08.10  get_current_user refuses a revoked jti and 403s a suspended user or
             suspended tenant.
  T10-08.7   otp_codes keyed by (phone, tenant_id): two tenants sharing a phone
             get independent codes, never overwriting.

Full suite 1264 passed / 0 failed (+2). SPRINT 8 COMPLETE: 10/10.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -6861,15 +6861,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I94" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I94" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J94" s="11" t="n"/>
       <c r="K94" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s8_isolation_scenarios.test_get_current_user_isolation_guards_present: the legacy no-membership fallback is trusted ONLY when the user's own tenant_id == the token's claimed tenant (source-pinned), so a mid-migration token can't cause tenant confusion.</t>
         </is>
       </c>
       <c r="L94" s="11" t="inlineStr">
@@ -7085,15 +7085,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I98" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I98" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J98" s="11" t="n"/>
       <c r="K98" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s8_isolation_scenarios.test_otp_is_keyed_by_phone_and_tenant: otp_codes are keyed by (phone, tenant_id); two tenants sharing a phone get INDEPENDENT rows, never overwriting.</t>
         </is>
       </c>
       <c r="L98" s="11" t="inlineStr">
@@ -7253,15 +7253,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I101" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I101" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J101" s="11" t="n"/>
       <c r="K101" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s8_isolation_scenarios.test_get_current_user_isolation_guards_present: get_current_user refuses a revoked jti (is_revoked) and 403s a suspended user or suspended tenant (source-pinned; is_revoked behavior covered in test_session_revocation).</t>
         </is>
       </c>
       <c r="L101" s="11" t="inlineStr">

</xml_diff>

<commit_message>
test(concurrency): Epic 10 Sprint 10 batch 1 -- CAS, webhook idempotency, auto-invoice race
  T10-10.1   8 concurrent stage_version CAS updates -> exactly 1 wins; single-
             writer contract holds at runtime.
  T10-10.10  5 concurrent duplicate billing webhooks -> only 1 accepted (unique
             index blocks double-charge/double-upgrade).
  T10-10.8   auto-invoice: serialized re-run never double-books (source_task_id
             guard); documented that the find-then-insert has no unique index so
             a true race could double-book.

Full suite 1267 passed / 0 failed (+3). Sprint 10 now 4/10.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -7981,15 +7981,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I114" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I114" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J114" s="11" t="n"/>
       <c r="K114" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s10_concurrency_scenarios.test_stage_version_cas_admits_exactly_one_writer: 8 concurrent stage_version CAS updates -&gt; exactly 1 wins (modified_count sums to 1), version advances exactly once. Single-writer contract holds at runtime.</t>
         </is>
       </c>
       <c r="L114" s="11" t="inlineStr">
@@ -8373,15 +8373,15 @@
           <t>S</t>
         </is>
       </c>
-      <c r="I121" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I121" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J121" s="11" t="n"/>
       <c r="K121" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s10_concurrency_scenarios.test_auto_invoice_concurrent_double_completion: a serialized re-run never double-books (source_task_id guard holds); documented that the find-then-insert guard has NO unique index, so a true race COULD double-book (1-or-2).</t>
         </is>
       </c>
       <c r="L121" s="11" t="inlineStr">
@@ -8485,15 +8485,15 @@
           <t>S</t>
         </is>
       </c>
-      <c r="I123" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I123" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J123" s="11" t="n"/>
       <c r="K123" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s10_concurrency_scenarios.test_billing_webhook_idempotency_key_is_unique: 5 concurrent duplicate webhooks -&gt; only 1 accepted, unique index blocks the rest (no double-charge/double-upgrade).</t>
         </is>
       </c>
       <c r="L123" s="11" t="inlineStr">

</xml_diff>

<commit_message>
test(concurrency): Epic 10 Sprint 10 -- seat-limit TOCTOU exposed (BUG-12)
  T10-10.3  worst-case interleaving (all invites run the cap CHECK before any
            INSERT) -> all 3 pass a cap of 3 with 2 used -> 5 active. Confirmed
            time-of-check/time-of-use over-provision: enforce_seat_limit is
            count-then-insert with no atomic reservation. Logged as BUG-12
            (fix = atomic seat reservation).

Full suite 1268 passed / 0 failed (+1). Sprint 10 now 5/10.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -8093,15 +8093,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I116" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I116" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J116" s="11" t="n"/>
       <c r="K116" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s10_concurrency_scenarios.test_seat_limit_toctou_over_provisions: worst-case interleaving (all invites run the cap CHECK before any INSERT) -&gt; all 3 pass a cap of 3 with 2 used -&gt; 5 active. CONFIRMED TOCTOU bug (BUG-12); needs an atomic seat reservation.</t>
         </is>
       </c>
       <c r="L116" s="11" t="inlineStr">
@@ -10305,7 +10305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11421,6 +11421,53 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>BUG-12</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>Billing / seats</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>enforce_seat_limit COUNTS active memberships then the caller INSERTS, with no atomic reservation between the two. Under concurrent invites at the cap boundary, every request passes the count (all see the same sub-cap number) and then commits -&gt; the workspace over-provisions past its plan's seat cap (proven: 5 active against a cap of 3).</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>Flagged (exposed by test; fix = atomic reservation -- e.g. a conditional findOneAndUpdate on a seat counter, or a unique (tenant,seat_index) reservation -- rather than count-then-insert).</t>
+        </is>
+      </c>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>test_s10_concurrency_scenarios.py</t>
+        </is>
+      </c>
+      <c r="I27" s="11" t="inlineStr">
+        <is>
+          <t>T10-10.3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test(concurrency): Epic 10 Sprint 10 batch 3 -- leader lock, quota overshoot, payment idempotency
  T10-10.6  5 replicas race the Mongo leader lock -> exactly 1 holds; holder can
            refresh; others refused while the lease is live.
  T10-10.5  two parallel check_quota(cost=60) vs cap 100 both pass -> collective
            overshoot (no reservation between check and spend).
  T10-10.9  standalone-payment expense: serialized re-run never double-books
            (payment_id guard); find-then-insert has no unique index (race gap).

Full suite 1271 passed / 0 failed (+3). Sprint 10 now 8/10.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -8205,15 +8205,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I118" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I118" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J118" s="11" t="n"/>
       <c r="K118" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s10_concurrency_scenarios.test_quota_overshoot_without_reservation: two parallel check_quota(cost=60) against a cap of 100 BOTH pass (each sees 0 used) -&gt; collectively burn 120, overshooting. No reservation between check and spend (fail-open aggregate).</t>
         </is>
       </c>
       <c r="L118" s="11" t="inlineStr">
@@ -8261,15 +8261,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I119" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I119" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J119" s="11" t="n"/>
       <c r="K119" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s10_concurrency_scenarios.test_leader_lock_elects_single_holder: 5 replicas try_acquire the same Mongo lock -&gt; exactly 1 wins; the holder can refresh its own lease; a different replica is refused while the lease is live (atomic leader election).</t>
         </is>
       </c>
       <c r="L119" s="11" t="inlineStr">
@@ -8429,15 +8429,15 @@
           <t>S</t>
         </is>
       </c>
-      <c r="I122" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I122" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J122" s="11" t="n"/>
       <c r="K122" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s10_concurrency_scenarios.test_standalone_payment_expense_idempotency: a serialized re-run never books a second expense (payment_id guard holds); documented that the find-then-insert on payment_id has no unique index so a true race could double-book.</t>
         </is>
       </c>
       <c r="L122" s="11" t="inlineStr">

</xml_diff>

<commit_message>
test(concurrency): finish Epic 10 Sprint 10 -- stage double-spawn (BUG-13) + throttle (10/10)
  T10-10.4  on_stage_enter find-then-insert on (workflow_id, stage_key) with no
            unique index -> concurrent re-entry double-spawns the template task
            (proven: 2). Logged as BUG-13 (fix = unique partial index / upsert).
  T10-10.7  the 60s follow-up throttle is a per-process in-memory dict (not shared
            across workers), so multi-worker can double-run -- but the escalation
            ladder's target<=escalation_level guard makes that idempotent/safe.

Full suite 1273 passed / 0 failed (+2). SPRINT 10 COMPLETE: 10/10.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic10_Testing.xlsx
+++ b/docs/DecisionOS_Epic10_Testing.xlsx
@@ -8149,15 +8149,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I117" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I117" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J117" s="11" t="n"/>
       <c r="K117" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s10_concurrency_scenarios.test_stage_enter_double_spawn_race: on_stage_enter is find-then-insert on (workflow_id, stage_key) with NO unique index -&gt; worst-case interleaving double-spawns the same template task (proven: 2). See BUG-13.</t>
         </is>
       </c>
       <c r="L117" s="11" t="inlineStr">
@@ -8317,15 +8317,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I120" s="11" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="I120" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="J120" s="11" t="n"/>
       <c r="K120" s="12" t="inlineStr">
         <is>
-          <t>Grounded in code map 2026-08-29</t>
+          <t>Done -- test_s10_concurrency_scenarios.test_followup_throttle_in_memory_and_escalation_idempotent: the 60s follow-up throttle is a per-process in-memory dict (not shared across workers), so a multi-worker deploy CAN double-run the sweep -- but the escalation ladder's target&lt;=escalation_level guard makes that safe (idempotent).</t>
         </is>
       </c>
       <c r="L120" s="11" t="inlineStr">
@@ -10305,7 +10305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11468,6 +11468,53 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>BUG-13</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Workflow engine / stage tasks</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>on_stage_enter spawns a stage's template tasks with a find({workflow_id,stage_key})-then-insert and NO unique index. A concurrent re-entry (an advance racing a retry, or two ticks) can pass the existence check together and both insert -&gt; duplicate template tasks at the stage (proven under worst-case interleaving).</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>Flagged (fix = a unique partial index on (tenant_id, workflow_id, stage_key, template) or an upsert on that key, instead of find-then-insert).</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H28" s="12" t="inlineStr">
+        <is>
+          <t>test_s10_concurrency_scenarios.py</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>T10-10.4</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>